<commit_message>
Expand workflow docs; add audit scripts & plan
Significant documentation and tooling updates: greatly expanded _application_workflow_diagram.md to a complete, 100% module/catalog-level architecture (updated date to 2026-05-21) with detailed core, chat drivers, agents, RAG, embeddings, and utilities breakdowns. Added a new design/plan note plans/20260521_http2_multistreaming_support.md describing HTTP/2 multistreaming support. Added audit scripts scripts/audit/update_xlsx_test_status.py and scripts/audit/verify_xlsx.py to automate updating and verifying XLSX test status files, and updated the binary test status spreadsheet Docs/Pruebas/MakerAI34_Test_Status_Feb_25_2026.xlsx accordingly.
</commit_message>
<xml_diff>
--- a/Docs/Pruebas/MakerAI34_Test_Status_Feb_25_2026.xlsx
+++ b/Docs/Pruebas/MakerAI34_Test_Status_Feb_25_2026.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A5:M17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -443,10 +443,6 @@
     <col width="8" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -887,7 +883,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -949,7 +945,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1078,7 +1074,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>OK (Gemma 4)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1108,7 +1104,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1150,7 +1146,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1222,7 +1218,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1289,7 +1285,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1329,7 +1325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1673,7 +1669,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>moonshot-v1-8k, moonshot-v1-32k-vision-preview</t>
+          <t>kimi-k2, kimi-k2.5 (was: moonshot-v1-8k, moonshot-v1-32k-vision-preview)</t>
         </is>
       </c>
     </row>
@@ -1742,6 +1738,125 @@
       <c r="C24" t="inlineStr">
         <is>
           <t>command-a-03-2025, command-a-reasoning-08-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Groq</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>TTS</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>canopylabs/orpheus-v1-english</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Groq</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Web Search</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>groq/compound, groq/compound-mini</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Groq</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Code Interpreter</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>groq/compound, groq/compound-mini</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ollama</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Audio STT</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>gemma4 (all 7 variants)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Mistral</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Audio STT</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>voxtral-mini-latest, voxtral-small-latest</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>LM Studio</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Vision</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>llama-3.2-11b-vision, gemma-3-4b/12b/27b</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>LM Studio</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Tools</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>llama-3.3-70b, qwen2.5-7b, mistral-7b, gemma-3-4b/12b/27b</t>
         </is>
       </c>
     </row>

</xml_diff>